<commit_message>
Created a new export listner
</commit_message>
<xml_diff>
--- a/testData/defectTabTestData/defectTestCaseTab_testData.xlsx
+++ b/testData/defectTabTestData/defectTestCaseTab_testData.xlsx
@@ -1,58 +1,67 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29905"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MohitAman\Desktop\UAT_NEXTNEXT_BLAZE_FRAMEWORK_AUTO\testData\defectTabTestData\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F90B0ED8-44F2-4604-A02D-5BDDBB7CABFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ECCB704D-C252-4BEE-B15E-93B86E1A650F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="16" activeTab="23" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="3" activeTab="30" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tc004" sheetId="4" r:id="rId1"/>
     <sheet name="tc006" sheetId="3" r:id="rId2"/>
     <sheet name="tc007" sheetId="8" r:id="rId3"/>
-    <sheet name="tc009" sheetId="1" r:id="rId4"/>
-    <sheet name="tc010" sheetId="2" r:id="rId5"/>
-    <sheet name="tc008" sheetId="29" r:id="rId6"/>
-    <sheet name="tc014" sheetId="6" r:id="rId7"/>
-    <sheet name="tc015" sheetId="7" r:id="rId8"/>
-    <sheet name="tc016" sheetId="9" r:id="rId9"/>
-    <sheet name="tc017" sheetId="10" r:id="rId10"/>
-    <sheet name="tc018" sheetId="17" r:id="rId11"/>
-    <sheet name="tc021" sheetId="11" r:id="rId12"/>
-    <sheet name="tc023" sheetId="12" r:id="rId13"/>
-    <sheet name="tc026" sheetId="15" r:id="rId14"/>
-    <sheet name="tc027" sheetId="20" r:id="rId15"/>
-    <sheet name="tc013" sheetId="26" r:id="rId16"/>
-    <sheet name="tc011" sheetId="30" r:id="rId17"/>
-    <sheet name="tc033" sheetId="27" r:id="rId18"/>
-    <sheet name="tc035" sheetId="28" r:id="rId19"/>
-    <sheet name="tc029" sheetId="13" r:id="rId20"/>
-    <sheet name="tc030" sheetId="14" r:id="rId21"/>
-    <sheet name="tc041" sheetId="16" r:id="rId22"/>
-    <sheet name="tc047" sheetId="18" r:id="rId23"/>
-    <sheet name="tc049" sheetId="31" r:id="rId24"/>
-    <sheet name="tc050" sheetId="32" r:id="rId25"/>
-    <sheet name="tc037" sheetId="24" r:id="rId26"/>
-    <sheet name="tc046" sheetId="19" r:id="rId27"/>
-    <sheet name="tc042" sheetId="23" r:id="rId28"/>
+    <sheet name="tc008" sheetId="29" r:id="rId4"/>
+    <sheet name="tc009" sheetId="1" r:id="rId5"/>
+    <sheet name="tc010" sheetId="2" r:id="rId6"/>
+    <sheet name="tc011" sheetId="30" r:id="rId7"/>
+    <sheet name="tc013" sheetId="26" r:id="rId8"/>
+    <sheet name="tc014" sheetId="6" r:id="rId9"/>
+    <sheet name="tc015" sheetId="7" r:id="rId10"/>
+    <sheet name="tc016" sheetId="9" r:id="rId11"/>
+    <sheet name="tc017" sheetId="10" r:id="rId12"/>
+    <sheet name="tc018" sheetId="17" r:id="rId13"/>
+    <sheet name="tc021" sheetId="11" r:id="rId14"/>
+    <sheet name="tc023" sheetId="12" r:id="rId15"/>
+    <sheet name="tc026" sheetId="15" r:id="rId16"/>
+    <sheet name="tc027" sheetId="20" r:id="rId17"/>
+    <sheet name="tc029" sheetId="13" r:id="rId18"/>
+    <sheet name="tc030" sheetId="14" r:id="rId19"/>
+    <sheet name="tc033" sheetId="27" r:id="rId20"/>
+    <sheet name="tc035" sheetId="28" r:id="rId21"/>
+    <sheet name="tc037" sheetId="24" r:id="rId22"/>
+    <sheet name="tc041" sheetId="16" r:id="rId23"/>
+    <sheet name="tc042" sheetId="23" r:id="rId24"/>
+    <sheet name="tc046" sheetId="19" r:id="rId25"/>
+    <sheet name="tc047" sheetId="18" r:id="rId26"/>
+    <sheet name="tc049" sheetId="32" r:id="rId27"/>
+    <sheet name="tc050" sheetId="31" r:id="rId28"/>
+    <sheet name="tc077" sheetId="33" r:id="rId29"/>
+    <sheet name="tc078" sheetId="34" r:id="rId30"/>
+    <sheet name="tc079" sheetId="35" r:id="rId31"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="94">
   <si>
     <t>project</t>
   </si>
@@ -108,6 +117,48 @@
     <t>DF-311</t>
   </si>
   <si>
+    <t>Affected_release</t>
+  </si>
+  <si>
+    <t>Severity</t>
+  </si>
+  <si>
+    <t>FixedR</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Module</t>
+  </si>
+  <si>
+    <t>Reason</t>
+  </si>
+  <si>
+    <t>Cat</t>
+  </si>
+  <si>
+    <t>target</t>
+  </si>
+  <si>
+    <t>SET- DRV</t>
+  </si>
+  <si>
+    <t>Minor</t>
+  </si>
+  <si>
+    <t>MD-297 SET- DRIV</t>
+  </si>
+  <si>
+    <t>Design - UI</t>
+  </si>
+  <si>
+    <t>Vivek Rajput</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
     <t>Summary</t>
   </si>
   <si>
@@ -120,46 +171,16 @@
     <t>Testing Description</t>
   </si>
   <si>
-    <t>Affected_release</t>
-  </si>
-  <si>
-    <t>Severity</t>
-  </si>
-  <si>
-    <t>FixedR</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Module</t>
-  </si>
-  <si>
-    <t>Reason</t>
-  </si>
-  <si>
-    <t>Cat</t>
-  </si>
-  <si>
-    <t>target</t>
-  </si>
-  <si>
-    <t>SET- DRV</t>
-  </si>
-  <si>
-    <t>Minor</t>
-  </si>
-  <si>
-    <t>MD-297 SET- DRIV</t>
-  </si>
-  <si>
-    <t>Design - UI</t>
-  </si>
-  <si>
-    <t>Vivek Rajput</t>
-  </si>
-  <si>
-    <t>Low</t>
+    <t>Summary123!@#</t>
+  </si>
+  <si>
+    <t>affectedRelease</t>
+  </si>
+  <si>
+    <t>assignTo</t>
+  </si>
+  <si>
+    <t>severity</t>
   </si>
   <si>
     <t>url</t>
@@ -284,7 +305,7 @@
 Steps to reproduce :
 Expected result :
 Actual result :
-User name : Mohit Aman
+User name : Julie Kumari
 Test data (if any) :
 Test case number : </t>
   </si>
@@ -298,18 +319,6 @@
 Test case number : </t>
   </si>
   <si>
-    <t>affectedRelease</t>
-  </si>
-  <si>
-    <t>assignTo</t>
-  </si>
-  <si>
-    <t>severity</t>
-  </si>
-  <si>
-    <t>Summary123!@#</t>
-  </si>
-  <si>
     <t>summary2</t>
   </si>
   <si>
@@ -322,6 +331,15 @@
     <t>assigned_To</t>
   </si>
   <si>
+    <t xml:space="preserve">status </t>
+  </si>
+  <si>
+    <t>testcase Summary</t>
+  </si>
+  <si>
+    <t>Automation Description</t>
+  </si>
+  <si>
     <t>ID</t>
   </si>
   <si>
@@ -337,16 +355,13 @@
     <t>&amp;&amp;&amp;&amp;</t>
   </si>
   <si>
-    <t xml:space="preserve">status </t>
-  </si>
-  <si>
-    <t>testcase Summary</t>
-  </si>
-  <si>
-    <t>Automation Description</t>
-  </si>
-  <si>
     <t>Creating defect notification 12-01-2026</t>
+  </si>
+  <si>
+    <t>Defect Id</t>
+  </si>
+  <si>
+    <t>DF-314</t>
   </si>
 </sst>
 </file>
@@ -371,7 +386,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -389,7 +404,7 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -843,7 +858,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DBB4210-9285-4E78-B062-C70F95124B52}">
   <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="34" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="7" t="s">
@@ -969,19 +984,132 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F176698D-2844-4849-825F-67D3B337053C}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultColWidth="29.42578125" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="5">
+        <v>1</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{172E0C13-61F9-4032-BF55-C665681D7995}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3D4B51D-576B-4DA1-BDAE-6F85096314D0}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="44.42578125" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="18.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>12</v>
+      </c>
+      <c r="H2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{79DE2057-255F-4088-8F5E-0E08F75750CC}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87E5D401-1490-449E-9C0A-3DF35853EE92}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="6" t="s">
         <v>14</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="C1" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -989,10 +1117,10 @@
         <v>16</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1003,14 +1131,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B310B858-FEFA-48A5-B995-DA133501E07F}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="6" max="6" width="14.453125" customWidth="1"/>
-    <col min="7" max="7" width="17.1796875" customWidth="1"/>
-    <col min="8" max="8" width="27.1796875" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" customWidth="1"/>
+    <col min="7" max="7" width="17.140625" customWidth="1"/>
+    <col min="8" max="8" width="27.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1018,25 +1146,25 @@
         <v>14</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="C1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="F1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="H1" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -1044,7 +1172,7 @@
         <v>16</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -1062,7 +1190,7 @@
         <v>12</v>
       </c>
       <c r="H2" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1073,28 +1201,28 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41609440-00B7-4122-9080-D2BC0A433D51}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="60.453125" customWidth="1"/>
+    <col min="2" max="2" width="60.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="116">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="115.5">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1105,10 +1233,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3259BD86-3F8F-4A42-86F4-5DD744C41E44}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="7" t="s">
@@ -1121,7 +1249,7 @@
         <v>6</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -1129,26 +1257,26 @@
         <v>7</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>13</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56806B28-3978-47F9-8A2E-A1FAB993CEA2}">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultColWidth="25.453125" defaultRowHeight="55.5" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="25.42578125" defaultRowHeight="55.5" customHeight="1"/>
   <cols>
-    <col min="1" max="16384" width="25.453125" style="11"/>
+    <col min="1" max="16384" width="25.42578125" style="11"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="55.5" customHeight="1">
@@ -1156,43 +1284,43 @@
         <v>0</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="M1" s="10" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="N1" s="10" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="55.5" customHeight="1">
@@ -1201,51 +1329,51 @@
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="12" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="G2" s="12" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="H2" s="12" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="I2" s="12" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="J2" s="12" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="K2" s="12" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="L2" s="12" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="M2" s="12" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>73</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>77</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8D2FA3B-A385-40DB-B8F7-3AD897BAF126}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="4" t="s">
@@ -1258,7 +1386,7 @@
         <v>6</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="105.75" customHeight="1">
@@ -1272,163 +1400,92 @@
         <v>13</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>74</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{484D8939-7FDB-49ED-81B6-808A8C8953E5}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="14.1796875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" ht="15">
-      <c r="A1" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAA3B7BB-8D47-428A-AFA2-8FBE09983B20}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="4" t="s">
+        <v>40</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>76</v>
+        <v>41</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="15">
-      <c r="A2" s="5">
-        <v>1</v>
-      </c>
-      <c r="B2" s="5">
-        <v>1</v>
-      </c>
-      <c r="C2" s="5">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{317972B3-61A5-430E-AD3E-E50EC8FDDA33}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="2" max="2" width="15.81640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" ht="15">
-      <c r="A1" s="5" t="s">
         <v>6</v>
       </c>
+      <c r="D1" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{37AC72DE-8FBE-4EDB-8A35-CE96D7521365}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{291E5E8B-3DC4-459B-886A-59328C11C1BB}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="4" t="s">
+        <v>40</v>
+      </c>
       <c r="B1" s="5" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="15">
-      <c r="A2" s="5">
-        <v>1</v>
+        <v>41</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="1" t="s">
+        <v>16</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{151DEB7C-D179-49F8-97B3-BE1831536417}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="14.7265625" customWidth="1"/>
-    <col min="4" max="4" width="28" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" ht="15">
-      <c r="A1" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="15">
-      <c r="A2" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="B2" s="5">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>81</v>
+        <v>13</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>80</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CC0CE84-E866-472B-BB42-2AAD8AE92A1A}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="14.7265625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" ht="15">
-      <c r="A1" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="15">
-      <c r="A2" s="5">
-        <v>2</v>
-      </c>
-      <c r="B2" s="5">
-        <v>1</v>
-      </c>
-      <c r="C2" s="5">
-        <v>1</v>
-      </c>
-      <c r="D2" s="5">
-        <v>2</v>
-      </c>
-      <c r="E2" s="5">
-        <v>5</v>
-      </c>
-    </row>
-  </sheetData>
+        <v>46</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{6784271E-276C-4D31-8375-14BA890EE7FF}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1436,7 +1493,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F11C9F18-0D54-4C96-BED8-DE87C1369977}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
@@ -1463,95 +1520,135 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAA3B7BB-8D47-428A-AFA2-8FBE09983B20}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{151DEB7C-D179-49F8-97B3-BE1831536417}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <sheetData>
-    <row r="1" spans="1:4" ht="15">
-      <c r="A1" s="4" t="s">
-        <v>36</v>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="3" max="3" width="19.42578125" customWidth="1"/>
+    <col min="4" max="4" width="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="5" t="s">
+        <v>32</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B2" s="5">
+        <v>1</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CC0CE84-E866-472B-BB42-2AAD8AE92A1A}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="5" t="s">
         <v>37</v>
       </c>
+      <c r="B1" s="5" t="s">
+        <v>6</v>
+      </c>
       <c r="C1" s="5" t="s">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="15">
-      <c r="A2" s="1" t="s">
-        <v>16</v>
+        <v>2</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="5">
+        <v>2</v>
+      </c>
+      <c r="B2" s="5">
+        <v>1</v>
+      </c>
+      <c r="C2" s="5">
+        <v>1</v>
+      </c>
+      <c r="D2" s="5">
+        <v>2</v>
+      </c>
+      <c r="E2" s="5">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5FD66FB-087A-4BE0-AD53-96903EBC09C4}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>39</v>
+        <v>13</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>42</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{37AC72DE-8FBE-4EDB-8A35-CE96D7521365}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{291E5E8B-3DC4-459B-886A-59328C11C1BB}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <sheetData>
-    <row r="1" spans="1:4" ht="15">
-      <c r="A1" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="15">
-      <c r="A2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>42</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{6784271E-276C-4D31-8375-14BA890EE7FF}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>85</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC29B807-E3D5-449A-8A03-0861456EF643}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="50.81640625" customWidth="1"/>
-    <col min="2" max="2" width="14.26953125" customWidth="1"/>
-    <col min="3" max="3" width="27.81640625" customWidth="1"/>
+    <col min="1" max="1" width="50.85546875" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" customWidth="1"/>
+    <col min="3" max="3" width="27.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1559,10 +1656,10 @@
         <v>14</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1570,10 +1667,10 @@
         <v>16</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -1584,37 +1681,113 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95CDEE87-BA4B-4159-A872-0FB688D1BFE4}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{67828866-220C-48B5-9D02-8AE8FB19356A}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDCD33EE-0A44-410C-8DC5-C065FBFA5F79}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultColWidth="43" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{4A93CEC8-FAC0-4D43-94E1-539353D8B566}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4399D2F9-CD9F-4056-81A4-75DF083A99E0}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <sheetData>
-    <row r="1" spans="1:4" ht="15">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:4">
       <c r="A1" s="4" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>6</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="15">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1625,21 +1798,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33047308-8012-48E2-8299-A58FC9BA8DD3}">
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74CC4233-2CFC-4966-950B-EC7D472B0249}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="33.36328125" customWidth="1"/>
-    <col min="2" max="2" width="36" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="B1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -1655,20 +1824,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94D4A305-01E5-424A-9C03-71CDEBB0FB71}">
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E13CA0E3-E524-4F3E-8155-BEFFD762B195}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="B1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1687,144 +1856,234 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5FD66FB-087A-4BE0-AD53-96903EBC09C4}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <sheetData>
-    <row r="1" spans="1:3" ht="15">
-      <c r="A1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="15">
-      <c r="A2" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>90</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDCD33EE-0A44-410C-8DC5-C065FBFA5F79}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="43" defaultRowHeight="14.5"/>
-  <sheetData>
-    <row r="1" spans="1:4" ht="15">
-      <c r="A1" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="15">
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67D6AC7E-4F3D-4BB7-9EBB-B637C55ECA43}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4800AC7E-F153-4191-9E90-3380C12B1430}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
       <c r="A2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C2" s="5" t="s">
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{98773125-5332-4379-98B8-0FD3F271177C}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{194BFBF1-4FAF-40AC-B8D4-3CC28997BD70}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7B18CC4-7FD5-4F7E-9DF8-133ED589EAF0}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF62085B-EB17-4E72-8097-DEB2C8E971B5}">
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr defaultColWidth="15" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="16384" width="15" style="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="G1" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="L1" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="M1" s="17" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="H2" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="I2" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="J2" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="K2" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="L2" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="5" t="s">
-        <v>42</v>
+      <c r="M2" s="17" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{4A93CEC8-FAC0-4D43-94E1-539353D8B566}"/>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{C2C43611-9FF1-4030-9070-7939D6470EEA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95CDEE87-BA4B-4159-A872-0FB688D1BFE4}">
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="41.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="7" t="s">
+      <c r="A1" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>18</v>
+      <c r="B1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="14" t="s">
-        <v>84</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>85</v>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{67828866-220C-48B5-9D02-8AE8FB19356A}"/>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{938664A6-98D0-4D67-82A6-5216F9BEBF97}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4800AC7E-F153-4191-9E90-3380C12B1430}">
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1">
-      <c r="A2" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{98773125-5332-4379-98B8-0FD3F271177C}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{984425FB-E0ED-4499-9F06-D56178AE2B8E}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="41.7265625" customWidth="1"/>
-    <col min="2" max="2" width="21.1796875" customWidth="1"/>
+    <col min="1" max="1" width="30.85546875" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="22.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1832,197 +2091,123 @@
         <v>14</v>
       </c>
       <c r="B1" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="C1" t="s">
-        <v>19</v>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{CFA4C855-DE38-4355-86BF-026061729869}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{317972B3-61A5-430E-AD3E-E50EC8FDDA33}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="15.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="5">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{484D8939-7FDB-49ED-81B6-808A8C8953E5}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="5">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5">
+        <v>1</v>
+      </c>
+      <c r="C2" s="5">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57C9431D-5367-4EBD-BB7D-638E4D59A5BF}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{938664A6-98D0-4D67-82A6-5216F9BEBF97}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{984425FB-E0ED-4499-9F06-D56178AE2B8E}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="45.453125" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="22.453125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{CFA4C855-DE38-4355-86BF-026061729869}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF62085B-EB17-4E72-8097-DEB2C8E971B5}">
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultColWidth="15" defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="16384" width="15" style="15"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="D1" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="F1" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="G1" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="17" t="s">
-        <v>28</v>
-      </c>
-      <c r="J1" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="K1" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="L1" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="M1" s="17" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="D2" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="E2" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="F2" s="17" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="H2" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="I2" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="J2" s="17" t="s">
-        <v>34</v>
-      </c>
-      <c r="K2" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="L2" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="M2" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{C2C43611-9FF1-4030-9070-7939D6470EEA}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57C9431D-5367-4EBD-BB7D-638E4D59A5BF}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="24.453125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" ht="15">
-      <c r="A1" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="15">
-      <c r="A2" s="1" t="s">
-        <v>16</v>
-      </c>
       <c r="B2" s="5" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -2031,117 +2216,4 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F176698D-2844-4849-825F-67D3B337053C}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="29.453125" defaultRowHeight="14.5"/>
-  <sheetData>
-    <row r="1" spans="1:4" ht="15">
-      <c r="A1" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="15">
-      <c r="A2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C2" s="5">
-        <v>1</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>42</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{172E0C13-61F9-4032-BF55-C665681D7995}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3D4B51D-576B-4DA1-BDAE-6F85096314D0}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="44.453125" customWidth="1"/>
-    <col min="2" max="2" width="15.54296875" customWidth="1"/>
-    <col min="4" max="4" width="20.1796875" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="18.26953125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8">
-      <c r="A1" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F1" t="s">
-        <v>45</v>
-      </c>
-      <c r="G1" t="s">
-        <v>46</v>
-      </c>
-      <c r="H1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>2</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>12</v>
-      </c>
-      <c r="H2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{79DE2057-255F-4088-8F5E-0E08F75750CC}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>